<commit_message>
No third-party branding: generic tools, official sources, ad windows aligned
Email tools, wallets, payment providers, AI assistants and spreadsheet
apps described generically in app copy, docs and guides; store check
names app kinds, not vendors; trend sources moved to official help pages
(two vendor-only trends dropped); vendor videos removed from the path;
SOP 06 and the compound plan judge ads on the 7-day window Helix reads,
with the 3-day MER check from Lesson 6.12; lead time wording aligned.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/downloads/helix-metrics-tracker.xlsx
+++ b/public/downloads/helix-metrics-tracker.xlsx
@@ -577,7 +577,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>Google Sheets: File &gt; Import &gt; Upload this file. Excel and Numbers open it directly.</t>
+          <t>Any spreadsheet app opens this file. In an online spreadsheet, use File &gt; Import &gt; Upload.</t>
         </is>
       </c>
     </row>
@@ -744,7 +744,7 @@
       </c>
       <c r="I2" s="4" t="inlineStr">
         <is>
-          <t>Shopify Payments, PayPal and so on</t>
+          <t>Shopify Payments and other payment providers</t>
         </is>
       </c>
       <c r="J2" s="4" t="inlineStr">

</xml_diff>